<commit_message>
feat: split PDF services & fix perincian data kuantitas layout - Split pdf_report_service into pdf_perincian_service, pdf_ringkasan_service, pdf_blank_service - Fix Nama KRT & Nama KK alignment (rata kiri) - Fix Jumlah row merge across columns 1-2-3 (rata tengah) - Fix header DATA KUANTITAS positioning above Nama Kepala Keluarga - Clean up 24 scratch scripts from root directory - Remove unused _parseInt and suppress unused tableHeaders warning - Zero issues on dart analyze
</commit_message>
<xml_diff>
--- a/data/database dawis 10.xlsx
+++ b/data/database dawis 10.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\DAWIS\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\DAWIS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59378356-E1C7-4A81-BC90-BBE98771F51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702C5B0B-CA71-4002-B0F9-B3CA20A0926F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6F9E1E13-26B6-44B5-AD04-A10CFD5709DA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="588">
   <si>
     <t>00.000.000.0-000.000</t>
   </si>
@@ -1256,57 +1256,18 @@
     <t>BUAH GOWOK 010.008.001</t>
   </si>
   <si>
-    <t>153.23.20501.3</t>
-  </si>
-  <si>
-    <t>martini 1957@ g email.com</t>
-  </si>
-  <si>
-    <t>085776784886</t>
-  </si>
-  <si>
     <t>Jl Nanas No.19 RT 007 / RW 010 Utan Kayu Utara, Matraman, Jakarta-Timur 13120</t>
   </si>
   <si>
-    <t>Jl Nanas No 19</t>
-  </si>
-  <si>
-    <t>Solo</t>
-  </si>
-  <si>
-    <t>3175016003570003</t>
-  </si>
-  <si>
     <t>T16478</t>
   </si>
   <si>
-    <t>SRI MARTINI</t>
-  </si>
-  <si>
     <t>BUAH GOWOK 010.007.002</t>
   </si>
   <si>
-    <t>citrayenni@gmail.com</t>
-  </si>
-  <si>
-    <t>085959313637</t>
-  </si>
-  <si>
     <t>Jl Nanas No 15 RT 007 / RW 010 Utan Kayu Utara, Matraman, Jakarta-Timur 13120</t>
   </si>
   <si>
-    <t xml:space="preserve">Jl Nanas No 15 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Padang </t>
-  </si>
-  <si>
-    <t>3175014909800013</t>
-  </si>
-  <si>
-    <t>CITRA YENNI</t>
-  </si>
-  <si>
     <t xml:space="preserve">sitimaemanati@gmail.com </t>
   </si>
   <si>
@@ -1809,6 +1770,36 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>FATIHA ALYSSA SULTON</t>
+  </si>
+  <si>
+    <t>3175015404050001</t>
+  </si>
+  <si>
+    <t>KEBUMEN</t>
+  </si>
+  <si>
+    <t>Jl Nanas No 24</t>
+  </si>
+  <si>
+    <t>087811042348</t>
+  </si>
+  <si>
+    <t>SITI FATIMAH NUR AISYAH</t>
+  </si>
+  <si>
+    <t>3175014712020007</t>
+  </si>
+  <si>
+    <t>JAKARTA</t>
+  </si>
+  <si>
+    <t>Jl Nanas No 16</t>
+  </si>
+  <si>
+    <t>085817222497</t>
   </si>
 </sst>
 </file>
@@ -2208,70 +2199,70 @@
   <sheetData>
     <row r="1" spans="1:22" s="12" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>590</v>
+        <v>577</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>589</v>
+        <v>576</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>587</v>
+        <v>574</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>586</v>
+        <v>573</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>585</v>
+        <v>572</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>584</v>
+        <v>571</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>583</v>
+        <v>570</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>582</v>
+        <v>569</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>581</v>
+        <v>568</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>580</v>
+        <v>567</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>579</v>
+        <v>566</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>578</v>
+        <v>565</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>577</v>
+        <v>564</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>576</v>
+        <v>563</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>575</v>
+        <v>562</v>
       </c>
       <c r="Q1" s="13" t="s">
-        <v>574</v>
+        <v>561</v>
       </c>
       <c r="R1" s="13" t="s">
-        <v>573</v>
+        <v>560</v>
       </c>
       <c r="S1" s="13" t="s">
-        <v>572</v>
+        <v>559</v>
       </c>
       <c r="T1" s="13" t="s">
-        <v>571</v>
+        <v>558</v>
       </c>
       <c r="U1" s="13" t="s">
-        <v>570</v>
+        <v>557</v>
       </c>
       <c r="V1" s="13" t="s">
-        <v>569</v>
+        <v>556</v>
       </c>
     </row>
     <row r="2" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2279,19 +2270,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>568</v>
+        <v>555</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>567</v>
+        <v>554</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>566</v>
+        <v>553</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>542</v>
+        <v>529</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>565</v>
+        <v>552</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>24</v>
@@ -2303,10 +2294,10 @@
         <v>12</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>564</v>
+        <v>551</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>542</v>
+        <v>529</v>
       </c>
       <c r="L2" s="9" t="s">
         <v>9</v>
@@ -2327,40 +2318,40 @@
         <v>5</v>
       </c>
       <c r="R2" s="7" t="s">
-        <v>563</v>
+        <v>550</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>562</v>
+        <v>549</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>561</v>
+        <v>548</v>
       </c>
       <c r="U2" s="6" t="s">
-        <v>560</v>
+        <v>547</v>
       </c>
       <c r="V2" s="6" t="s">
-        <v>559</v>
+        <v>546</v>
       </c>
     </row>
     <row r="3" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
-        <f>A2+1</f>
+        <f t="shared" ref="A3:A34" si="0">A2+1</f>
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>558</v>
+        <v>545</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>557</v>
+        <v>544</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>556</v>
+        <v>543</v>
       </c>
       <c r="E3" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>542</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>555</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>117</v>
@@ -2372,10 +2363,10 @@
         <v>12</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>554</v>
+        <v>541</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>542</v>
+        <v>529</v>
       </c>
       <c r="L3" s="9" t="s">
         <v>9</v>
@@ -2396,40 +2387,40 @@
         <v>67</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>553</v>
+        <v>540</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>552</v>
+        <v>539</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>551</v>
+        <v>538</v>
       </c>
       <c r="U3" s="6" t="s">
-        <v>550</v>
+        <v>537</v>
       </c>
       <c r="V3" s="6" t="s">
-        <v>549</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11">
-        <f>A3+1</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>548</v>
+        <v>535</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>547</v>
+        <v>534</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>546</v>
+        <v>533</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>542</v>
+        <v>529</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>545</v>
+        <v>532</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>24</v>
@@ -2438,13 +2429,13 @@
         <v>28656</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>544</v>
+        <v>531</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>543</v>
+        <v>530</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>542</v>
+        <v>529</v>
       </c>
       <c r="L4" s="9" t="s">
         <v>9</v>
@@ -2465,16 +2456,16 @@
         <v>67</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>541</v>
+        <v>528</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>540</v>
+        <v>527</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>539</v>
+        <v>526</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>538</v>
+        <v>525</v>
       </c>
       <c r="V4" s="6" t="s">
         <v>52</v>
@@ -2482,23 +2473,23 @@
     </row>
     <row r="5" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11">
-        <f>A4+1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>537</v>
+        <v>524</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>536</v>
+        <v>523</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>535</v>
+        <v>522</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>534</v>
+        <v>521</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>24</v>
@@ -2510,10 +2501,10 @@
         <v>12</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>533</v>
+        <v>520</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>9</v>
@@ -2534,40 +2525,40 @@
         <v>67</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>532</v>
+        <v>519</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>531</v>
+        <v>518</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>530</v>
+        <v>517</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>529</v>
+        <v>516</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>528</v>
+        <v>515</v>
       </c>
     </row>
     <row r="6" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11">
-        <f>A5+1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>527</v>
+        <v>514</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>526</v>
+        <v>513</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>525</v>
+        <v>512</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>524</v>
+        <v>511</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>24</v>
@@ -2579,10 +2570,10 @@
         <v>12</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>523</v>
+        <v>510</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>9</v>
@@ -2603,16 +2594,16 @@
         <v>33</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>522</v>
+        <v>509</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>521</v>
+        <v>508</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>520</v>
+        <v>507</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>519</v>
+        <v>506</v>
       </c>
       <c r="V6" s="6" t="s">
         <v>52</v>
@@ -2620,23 +2611,23 @@
     </row>
     <row r="7" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11">
-        <f>A6+1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>518</v>
+        <v>505</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>517</v>
+        <v>504</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>516</v>
+        <v>503</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>515</v>
+        <v>502</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>24</v>
@@ -2648,10 +2639,10 @@
         <v>12</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>514</v>
+        <v>501</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>9</v>
@@ -2672,16 +2663,16 @@
         <v>5</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>512</v>
+        <v>499</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>511</v>
+        <v>498</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>510</v>
+        <v>497</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>509</v>
+        <v>496</v>
       </c>
       <c r="V7" s="6" t="s">
         <v>52</v>
@@ -2689,26 +2680,26 @@
     </row>
     <row r="8" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11">
-        <f>A7+1</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>508</v>
+        <v>495</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>507</v>
+        <v>494</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>506</v>
+        <v>493</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>493</v>
+        <v>480</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>505</v>
+        <v>492</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>504</v>
+        <v>491</v>
       </c>
       <c r="H8" s="10">
         <v>27180</v>
@@ -2717,10 +2708,10 @@
         <v>116</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>503</v>
+        <v>490</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>493</v>
+        <v>480</v>
       </c>
       <c r="L8" s="9" t="s">
         <v>9</v>
@@ -2741,16 +2732,16 @@
         <v>5</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>502</v>
+        <v>489</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>501</v>
+        <v>488</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>500</v>
+        <v>487</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>499</v>
+        <v>486</v>
       </c>
       <c r="V8" s="6" t="s">
         <v>52</v>
@@ -2758,23 +2749,23 @@
     </row>
     <row r="9" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <f>A8+1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>498</v>
+        <v>485</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>497</v>
+        <v>484</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>496</v>
+        <v>483</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>493</v>
+        <v>480</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>495</v>
+        <v>482</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>24</v>
@@ -2786,10 +2777,10 @@
         <v>12</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>494</v>
+        <v>481</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>493</v>
+        <v>480</v>
       </c>
       <c r="L9" s="9" t="s">
         <v>9</v>
@@ -2810,16 +2801,16 @@
         <v>33</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>492</v>
+        <v>479</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>491</v>
+        <v>478</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>490</v>
+        <v>477</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>489</v>
+        <v>476</v>
       </c>
       <c r="V9" s="6" t="s">
         <v>52</v>
@@ -2827,23 +2818,23 @@
     </row>
     <row r="10" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11">
-        <f>A9+1</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>488</v>
+        <v>475</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>487</v>
+        <v>474</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>473</v>
+        <v>460</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>485</v>
+        <v>472</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>24</v>
@@ -2855,10 +2846,10 @@
         <v>12</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>484</v>
+        <v>471</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>473</v>
+        <v>460</v>
       </c>
       <c r="L10" s="9" t="s">
         <v>9</v>
@@ -2879,16 +2870,16 @@
         <v>5</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>483</v>
+        <v>470</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>482</v>
+        <v>469</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>481</v>
+        <v>468</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="V10" s="6" t="s">
         <v>52</v>
@@ -2896,23 +2887,23 @@
     </row>
     <row r="11" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <f>A10+1</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>479</v>
+        <v>466</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>478</v>
+        <v>465</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>477</v>
+        <v>464</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>473</v>
+        <v>460</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>476</v>
+        <v>463</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>24</v>
@@ -2921,13 +2912,13 @@
         <v>27189</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>475</v>
+        <v>462</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>474</v>
+        <v>461</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>473</v>
+        <v>460</v>
       </c>
       <c r="L11" s="9" t="s">
         <v>9</v>
@@ -2948,16 +2939,16 @@
         <v>5</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>472</v>
+        <v>459</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>471</v>
+        <v>458</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>470</v>
+        <v>457</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>469</v>
+        <v>456</v>
       </c>
       <c r="V11" s="6" t="s">
         <v>52</v>
@@ -2965,23 +2956,23 @@
     </row>
     <row r="12" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11">
-        <f>A11+1</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>468</v>
+        <v>455</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>467</v>
+        <v>454</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>453</v>
+        <v>440</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>465</v>
+        <v>452</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>24</v>
@@ -2993,10 +2984,10 @@
         <v>116</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>464</v>
+        <v>451</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>453</v>
+        <v>440</v>
       </c>
       <c r="L12" s="9" t="s">
         <v>9</v>
@@ -3017,40 +3008,40 @@
         <v>5</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>463</v>
+        <v>450</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>462</v>
+        <v>449</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>461</v>
+        <v>448</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>460</v>
+        <v>447</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>459</v>
+        <v>446</v>
       </c>
     </row>
     <row r="13" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <f>A12+1</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>458</v>
+        <v>445</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>457</v>
+        <v>444</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>453</v>
+        <v>440</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>455</v>
+        <v>442</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>298</v>
@@ -3062,10 +3053,10 @@
         <v>58</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>454</v>
+        <v>441</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>453</v>
+        <v>440</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>9</v>
@@ -3086,31 +3077,31 @@
         <v>5</v>
       </c>
       <c r="R13" s="7" t="s">
-        <v>452</v>
+        <v>439</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>451</v>
+        <v>438</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>450</v>
+        <v>437</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>449</v>
+        <v>436</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>448</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11">
-        <f>A13+1</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>51</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>447</v>
+        <v>434</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>49</v>
@@ -3119,10 +3110,10 @@
         <v>45</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>446</v>
+        <v>433</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>445</v>
+        <v>432</v>
       </c>
       <c r="H14" s="10">
         <v>27565</v>
@@ -3131,7 +3122,7 @@
         <v>139</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>444</v>
+        <v>431</v>
       </c>
       <c r="K14" s="6" t="s">
         <v>45</v>
@@ -3155,13 +3146,13 @@
         <v>261</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>443</v>
+        <v>430</v>
       </c>
       <c r="S14" s="6" t="s">
-        <v>442</v>
+        <v>429</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>441</v>
+        <v>428</v>
       </c>
       <c r="U14" s="6" t="s">
         <v>221</v>
@@ -3172,23 +3163,23 @@
     </row>
     <row r="15" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11">
-        <f>A14+1</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>440</v>
+        <v>427</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>439</v>
+        <v>426</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>438</v>
+        <v>425</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>45</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>437</v>
+        <v>424</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>24</v>
@@ -3200,7 +3191,7 @@
         <v>58</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>436</v>
+        <v>423</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>45</v>
@@ -3224,16 +3215,16 @@
         <v>67</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>434</v>
+        <v>421</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>433</v>
+        <v>420</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>432</v>
+        <v>419</v>
       </c>
       <c r="V15" s="6" t="s">
         <v>52</v>
@@ -3241,26 +3232,26 @@
     </row>
     <row r="16" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11">
-        <f>A15+1</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>431</v>
+        <v>418</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>430</v>
+        <v>417</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>429</v>
+        <v>416</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>45</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>428</v>
+        <v>415</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>427</v>
+        <v>414</v>
       </c>
       <c r="H16" s="10">
         <v>25666</v>
@@ -3269,7 +3260,7 @@
         <v>116</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>426</v>
+        <v>413</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>45</v>
@@ -3293,13 +3284,13 @@
         <v>5</v>
       </c>
       <c r="R16" s="7" t="s">
-        <v>425</v>
+        <v>412</v>
       </c>
       <c r="S16" s="6" t="s">
-        <v>424</v>
+        <v>411</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>423</v>
+        <v>410</v>
       </c>
       <c r="U16" s="6" t="s">
         <v>221</v>
@@ -3310,14 +3301,14 @@
     </row>
     <row r="17" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11">
-        <f>A16+1</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>62</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>422</v>
+        <v>578</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>60</v>
@@ -3326,19 +3317,19 @@
         <v>56</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>421</v>
+        <v>579</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>420</v>
+        <v>580</v>
       </c>
       <c r="H17" s="10">
-        <v>29473</v>
+        <v>38456</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>116</v>
+        <v>12</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>419</v>
+        <v>581</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>56</v>
@@ -3362,14 +3353,12 @@
         <v>5</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>417</v>
-      </c>
-      <c r="T17" s="6" t="s">
-        <v>416</v>
-      </c>
+        <v>582</v>
+      </c>
+      <c r="T17" s="6"/>
       <c r="U17" s="6" t="s">
         <v>221</v>
       </c>
@@ -3379,35 +3368,35 @@
     </row>
     <row r="18" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <f>A17+1</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>414</v>
+        <v>583</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>56</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>412</v>
+        <v>584</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>411</v>
+        <v>585</v>
       </c>
       <c r="H18" s="10">
-        <v>20899</v>
+        <v>37263</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>410</v>
+        <v>586</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>56</v>
@@ -3431,16 +3420,14 @@
         <v>5</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="T18" s="6" t="s">
-        <v>407</v>
-      </c>
+        <v>587</v>
+      </c>
+      <c r="T18" s="6"/>
       <c r="U18" s="6" t="s">
-        <v>406</v>
+        <v>221</v>
       </c>
       <c r="V18" s="6" t="s">
         <v>52</v>
@@ -3448,7 +3435,7 @@
     </row>
     <row r="19" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="11">
-        <f>A18+1</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -3517,7 +3504,7 @@
     </row>
     <row r="20" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
-        <f>A19+1</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -3586,7 +3573,7 @@
     </row>
     <row r="21" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="11">
-        <f>A20+1</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -3655,7 +3642,7 @@
     </row>
     <row r="22" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="11">
-        <f>A21+1</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -3724,7 +3711,7 @@
     </row>
     <row r="23" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <f>A22+1</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -3793,7 +3780,7 @@
     </row>
     <row r="24" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
-        <f>A23+1</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -3862,7 +3849,7 @@
     </row>
     <row r="25" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <f>A24+1</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
@@ -3931,7 +3918,7 @@
     </row>
     <row r="26" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
-        <f>A25+1</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="B26" s="6" t="s">
@@ -4000,7 +3987,7 @@
     </row>
     <row r="27" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <f>A26+1</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
@@ -4069,7 +4056,7 @@
     </row>
     <row r="28" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="11">
-        <f>A27+1</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -4138,7 +4125,7 @@
     </row>
     <row r="29" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <f>A28+1</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -4207,7 +4194,7 @@
     </row>
     <row r="30" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="11">
-        <f>A29+1</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="B30" s="6" t="s">
@@ -4276,7 +4263,7 @@
     </row>
     <row r="31" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <f>A30+1</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
@@ -4345,7 +4332,7 @@
     </row>
     <row r="32" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="11">
-        <f>A31+1</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
@@ -4414,7 +4401,7 @@
     </row>
     <row r="33" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="11">
-        <f>A32+1</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -4483,7 +4470,7 @@
     </row>
     <row r="34" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="11">
-        <f>A33+1</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
@@ -4552,7 +4539,7 @@
     </row>
     <row r="35" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="11">
-        <f>A34+1</f>
+        <f t="shared" ref="A35:A59" si="1">A34+1</f>
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -4621,7 +4608,7 @@
     </row>
     <row r="36" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <f>A35+1</f>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -4690,7 +4677,7 @@
     </row>
     <row r="37" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="11">
-        <f>A36+1</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -4759,7 +4746,7 @@
     </row>
     <row r="38" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <f>A37+1</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -4828,7 +4815,7 @@
     </row>
     <row r="39" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="11">
-        <f>A38+1</f>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -4897,7 +4884,7 @@
     </row>
     <row r="40" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="11">
-        <f>A39+1</f>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -4966,7 +4953,7 @@
     </row>
     <row r="41" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="11">
-        <f>A40+1</f>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -5035,7 +5022,7 @@
     </row>
     <row r="42" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="11">
-        <f>A41+1</f>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -5104,7 +5091,7 @@
     </row>
     <row r="43" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <f>A42+1</f>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -5173,7 +5160,7 @@
     </row>
     <row r="44" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="11">
-        <f>A43+1</f>
+        <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -5242,7 +5229,7 @@
     </row>
     <row r="45" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <f>A44+1</f>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
@@ -5311,7 +5298,7 @@
     </row>
     <row r="46" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="11">
-        <f>A45+1</f>
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -5380,7 +5367,7 @@
     </row>
     <row r="47" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="11">
-        <f>A46+1</f>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
@@ -5449,7 +5436,7 @@
     </row>
     <row r="48" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="11">
-        <f>A47+1</f>
+        <f t="shared" si="1"/>
         <v>47</v>
       </c>
       <c r="B48" s="6" t="s">
@@ -5518,7 +5505,7 @@
     </row>
     <row r="49" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="11">
-        <f>A48+1</f>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
@@ -5587,7 +5574,7 @@
     </row>
     <row r="50" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <f>A49+1</f>
+        <f t="shared" si="1"/>
         <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
@@ -5656,7 +5643,7 @@
     </row>
     <row r="51" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="11">
-        <f>A50+1</f>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="B51" s="6" t="s">
@@ -5725,7 +5712,7 @@
     </row>
     <row r="52" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <f>A51+1</f>
+        <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
@@ -5794,7 +5781,7 @@
     </row>
     <row r="53" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="11">
-        <f>A52+1</f>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
@@ -5863,7 +5850,7 @@
     </row>
     <row r="54" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="11">
-        <f>A53+1</f>
+        <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
@@ -5932,7 +5919,7 @@
     </row>
     <row r="55" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="11">
-        <f>A54+1</f>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
@@ -6001,7 +5988,7 @@
     </row>
     <row r="56" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="11">
-        <f>A55+1</f>
+        <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="B56" s="6" t="s">
@@ -6070,7 +6057,7 @@
     </row>
     <row r="57" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <f>A56+1</f>
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
@@ -6139,7 +6126,7 @@
     </row>
     <row r="58" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="11">
-        <f>A57+1</f>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="B58" s="6" t="s">
@@ -6208,7 +6195,7 @@
     </row>
     <row r="59" spans="1:22" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <f>A58+1</f>
+        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="B59" s="6" t="s">

</xml_diff>